<commit_message>
docs: organizacion de artefactos de qa y documentacion
</commit_message>
<xml_diff>
--- a/qa/Métricas/Dashboard QA.xlsx
+++ b/qa/Métricas/Dashboard QA.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Dashboard" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="P-QA-13 Dashboard" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="Datos CP" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="Bugs" sheetId="3" r:id="rId6"/>
   </sheets>
@@ -11,14 +11,53 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="KduS4w1nrYmOKhNXACacqmV0MtggxEwwVyzC/36bEvY="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="EBeKFlyJspZgjedYQ4rhBy255RZ6ayKz/OOWNt5wXTE="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="E36">
+      <text>
+        <t xml:space="preserve">======
+ID#AAACFyDGtQw
+camila mahecha    (2026-08-19 19:30:33)
+CP-012(todo)</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="E31">
+      <text>
+        <t xml:space="preserve">======
+ID#AAACFyDGtQ0
+camila mahecha    (2026-08-19 19:31:15)
+CP-006(todo)</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="G31">
+      <text>
+        <t xml:space="preserve">======
+ID#AAACFyDGtQs
+camila mahecha    (2026-08-19 19:29:32)
+CP-006 (todo)</t>
+      </text>
+    </comment>
+  </commentList>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mi+J/N1xbBsyb7Km/iYwmH4beXnqQ=="/>
+    </ext>
+  </extLst>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="86">
   <si>
     <t>EP</t>
   </si>
@@ -29,87 +68,108 @@
     <t>Prioridad</t>
   </si>
   <si>
+    <t>Total CP</t>
+  </si>
+  <si>
+    <t>Unitaria - Ejecutados</t>
+  </si>
+  <si>
+    <t>Unitaria - Pasan</t>
+  </si>
+  <si>
+    <t>Integracion - Ejecutados</t>
+  </si>
+  <si>
+    <t>RF Completos (documentacion)</t>
+  </si>
+  <si>
+    <t>Integracion - Pasan</t>
+  </si>
+  <si>
     <t>Severidad</t>
   </si>
   <si>
-    <t>Total CP</t>
+    <t>Manual - Ejecutados</t>
+  </si>
+  <si>
+    <t>Manual - Pasan</t>
   </si>
   <si>
     <t>Cantidad Abiertos</t>
   </si>
   <si>
-    <t>Unitaria - Ejecutados</t>
-  </si>
-  <si>
     <t>Alta</t>
   </si>
   <si>
-    <t>Unitaria - Pasan</t>
-  </si>
-  <si>
-    <t>RF Completos (documentacion)</t>
-  </si>
-  <si>
-    <t>Integracion - Ejecutados</t>
-  </si>
-  <si>
     <t>Media</t>
   </si>
   <si>
-    <t>Integracion - Pasan</t>
+    <t>EP-001</t>
+  </si>
+  <si>
+    <t>Total CP definidos</t>
   </si>
   <si>
     <t>Baja</t>
   </si>
   <si>
-    <t>Manual - Ejecutados</t>
-  </si>
-  <si>
-    <t>Total CP definidos</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Manual - Pasan</t>
-  </si>
-  <si>
     <t>Bugs abiertos</t>
   </si>
   <si>
-    <t>CP faltante Unitarias</t>
-  </si>
-  <si>
-    <t>CP faltante Integración</t>
-  </si>
-  <si>
-    <t>CP fallo Manual</t>
-  </si>
-  <si>
-    <t>EP-001</t>
-  </si>
-  <si>
     <t>RF-001.1</t>
   </si>
   <si>
+    <t>RF-001.2</t>
+  </si>
+  <si>
+    <t>RF-001.3</t>
+  </si>
+  <si>
+    <t>RF-001.4</t>
+  </si>
+  <si>
+    <t>RF-001.5</t>
+  </si>
+  <si>
+    <t>RF-001.6</t>
+  </si>
+  <si>
+    <t>RF-001.7</t>
+  </si>
+  <si>
     <t>Informe Checklist</t>
   </si>
   <si>
+    <t>RF-001.8</t>
+  </si>
+  <si>
     <t>Checklist QA</t>
   </si>
   <si>
+    <t>EP-002</t>
+  </si>
+  <si>
     <t>Reporte de Bugs</t>
   </si>
   <si>
-    <t>RF-001.2</t>
+    <t>RF-002.1</t>
   </si>
   <si>
     <t>Avance de Ejecucion por Tipo de Prueba</t>
   </si>
   <si>
+    <t>RF-002.2</t>
+  </si>
+  <si>
     <t>Tipo de Prueba</t>
   </si>
   <si>
+    <t>RF-002.3</t>
+  </si>
+  <si>
     <t>CP Ejecutados</t>
   </si>
   <si>
@@ -122,27 +182,87 @@
     <t>% Aprobados (de ejecutados)</t>
   </si>
   <si>
+    <t>RF-002.4</t>
+  </si>
+  <si>
     <t>Unitaria</t>
   </si>
   <si>
-    <t>RF-001.3</t>
+    <t>RF-002.5</t>
+  </si>
+  <si>
+    <t>EP-003</t>
+  </si>
+  <si>
+    <t>RF-003.1</t>
+  </si>
+  <si>
+    <t>RF-003.2</t>
+  </si>
+  <si>
+    <t>RF-003.3</t>
+  </si>
+  <si>
+    <t>RF-003.4</t>
+  </si>
+  <si>
+    <t>EP-004</t>
+  </si>
+  <si>
+    <t>RF-004.1</t>
+  </si>
+  <si>
+    <t>RF-004.2</t>
+  </si>
+  <si>
+    <t>RF-004.3</t>
+  </si>
+  <si>
+    <t>RF-004.4</t>
+  </si>
+  <si>
+    <t>EP-005</t>
+  </si>
+  <si>
+    <t>RF-005.1</t>
   </si>
   <si>
     <t>Integracion</t>
   </si>
   <si>
-    <t>RF-001.4</t>
+    <t>RF-005.2</t>
+  </si>
+  <si>
+    <t>EP-006</t>
+  </si>
+  <si>
+    <t>RF-006.1</t>
   </si>
   <si>
     <t>Manual</t>
   </si>
   <si>
-    <t>RF-001.5</t>
+    <t>RF-006.2</t>
+  </si>
+  <si>
+    <t>RF-006.3</t>
+  </si>
+  <si>
+    <t>RF-006.4</t>
+  </si>
+  <si>
+    <t>RF-006.5</t>
+  </si>
+  <si>
+    <t>EP-007</t>
   </si>
   <si>
     <t>Avance de Ejecucion por Prioridad (vs. Meta del Plan Maestro)</t>
   </si>
   <si>
+    <t>RF-007.1</t>
+  </si>
+  <si>
     <t>Meta</t>
   </si>
   <si>
@@ -152,175 +272,49 @@
     <t>Integracion %</t>
   </si>
   <si>
+    <t>RF-007.2</t>
+  </si>
+  <si>
     <t>Manual %</t>
   </si>
   <si>
     <t>Cumple Meta</t>
   </si>
   <si>
-    <t>RF-001.6</t>
-  </si>
-  <si>
-    <t>RF-001.7</t>
-  </si>
-  <si>
-    <t>RF-001.8</t>
-  </si>
-  <si>
-    <t>EP-002</t>
-  </si>
-  <si>
-    <t>RF-002.1</t>
-  </si>
-  <si>
-    <t>RF-002.2</t>
-  </si>
-  <si>
-    <t>RF-002.3</t>
-  </si>
-  <si>
-    <t>RF-002.4</t>
-  </si>
-  <si>
-    <t>RF-002.5</t>
-  </si>
-  <si>
-    <t>EP-003</t>
-  </si>
-  <si>
-    <t>RF-003.1</t>
+    <t>RF-007.3</t>
+  </si>
+  <si>
+    <t>EP-008</t>
+  </si>
+  <si>
+    <t>RF-008.1</t>
+  </si>
+  <si>
+    <t>RF-008.2</t>
+  </si>
+  <si>
+    <t>RF-008.3</t>
+  </si>
+  <si>
+    <t>RF-008.4</t>
+  </si>
+  <si>
+    <t>EP-009</t>
+  </si>
+  <si>
+    <t>RF-009.1</t>
+  </si>
+  <si>
+    <t>RF-009.2</t>
+  </si>
+  <si>
+    <t>RF-009.3</t>
   </si>
   <si>
     <t>Bugs Abiertos por Severidad</t>
   </si>
   <si>
     <t>Cantidad</t>
-  </si>
-  <si>
-    <t>RF-003.2</t>
-  </si>
-  <si>
-    <t>RF-003.3</t>
-  </si>
-  <si>
-    <t>RF-003.4</t>
-  </si>
-  <si>
-    <t>EP-004</t>
-  </si>
-  <si>
-    <t>RF-004.1</t>
-  </si>
-  <si>
-    <t>RF-004.2</t>
-  </si>
-  <si>
-    <t>RF-004.3</t>
-  </si>
-  <si>
-    <t>RF-004.4</t>
-  </si>
-  <si>
-    <t>EP-005</t>
-  </si>
-  <si>
-    <t>RF-005.1</t>
-  </si>
-  <si>
-    <t>CP-001, CP-002</t>
-  </si>
-  <si>
-    <t>Todos</t>
-  </si>
-  <si>
-    <t>CP-004 (BUG-007)</t>
-  </si>
-  <si>
-    <t>RF-005.2</t>
-  </si>
-  <si>
-    <t>EP-006</t>
-  </si>
-  <si>
-    <t>RF-006.1</t>
-  </si>
-  <si>
-    <t>RF-006.2</t>
-  </si>
-  <si>
-    <t>RF-006.3</t>
-  </si>
-  <si>
-    <t>RF-006.4</t>
-  </si>
-  <si>
-    <t>RF-006.5</t>
-  </si>
-  <si>
-    <t>EP-007</t>
-  </si>
-  <si>
-    <t>RF-007.1</t>
-  </si>
-  <si>
-    <t>CP-004</t>
-  </si>
-  <si>
-    <t>RF-007.2</t>
-  </si>
-  <si>
-    <t>CP-008</t>
-  </si>
-  <si>
-    <t>CP-005 (BUG-008) CP-006 (BUG-009)</t>
-  </si>
-  <si>
-    <t>RF-007.3</t>
-  </si>
-  <si>
-    <t>CP-009 (BUG-0010), CP-010 (BUG-0011)</t>
-  </si>
-  <si>
-    <t>EP-008</t>
-  </si>
-  <si>
-    <t>RF-008.1</t>
-  </si>
-  <si>
-    <t>CP-002, CP-004</t>
-  </si>
-  <si>
-    <t>RF-008.2</t>
-  </si>
-  <si>
-    <t>CP-005 (BUG-012)</t>
-  </si>
-  <si>
-    <t>RF-008.3</t>
-  </si>
-  <si>
-    <t>RF-008.4</t>
-  </si>
-  <si>
-    <t>CP-011, CP-012</t>
-  </si>
-  <si>
-    <t>EP-009</t>
-  </si>
-  <si>
-    <t>RF-009.1</t>
-  </si>
-  <si>
-    <t>CP-003 (BUG-013)</t>
-  </si>
-  <si>
-    <t>RF-009.2</t>
-  </si>
-  <si>
-    <t>CP-005 (BUG-0014)</t>
-  </si>
-  <si>
-    <t>RF-009.3</t>
   </si>
 </sst>
 </file>
@@ -330,7 +324,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -362,17 +356,27 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
     <font/>
+    <font>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <b/>
       <sz val="14.0"/>
@@ -381,11 +385,6 @@
     </font>
     <font>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <color rgb="FF666666"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -407,7 +406,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -426,14 +425,8 @@
         <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC27BA0"/>
-        <bgColor rgb="FFC27BA0"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border/>
     <border>
       <left style="thin">
@@ -484,20 +477,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFB7B7B7"/>
       </left>
       <right style="thin">
@@ -519,7 +498,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -535,80 +514,74 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+    <xf borderId="5" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="7" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -864,155 +837,155 @@
       <c r="J3" s="2"/>
     </row>
     <row r="5" ht="15.0" customHeight="1">
-      <c r="B5" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="E5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="H5" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="8"/>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="E5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="9"/>
+      <c r="H5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="9"/>
     </row>
     <row r="6">
-      <c r="B6" s="11" t="str">
+      <c r="B6" s="15" t="str">
         <f>"38 / 38 (100%)"</f>
         <v>38 / 38 (100%)</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="11">
+      <c r="C6" s="9"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="15">
         <f>'Datos CP'!D40</f>
         <v>169</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="11">
+      <c r="F6" s="9"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="15">
         <f>Bugs!B8</f>
         <v>14</v>
       </c>
-      <c r="I6" s="8"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="B7" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="E7" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="H7" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" s="8"/>
+      <c r="B7" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="E7" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="H7" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="9"/>
     </row>
     <row r="10">
       <c r="B10" s="21" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="5">
+      <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="6">
         <f>'Datos CP'!D40</f>
         <v>169</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="6">
         <f>'Datos CP'!E40</f>
-        <v>60</v>
+        <v>131</v>
       </c>
       <c r="E12" s="22">
         <f t="shared" ref="E12:E14" si="1">IFERROR(D12/C12,0)</f>
-        <v>0.3550295858</v>
-      </c>
-      <c r="F12" s="5">
+        <v>0.775147929</v>
+      </c>
+      <c r="F12" s="6">
         <f>'Datos CP'!F40</f>
-        <v>53</v>
+        <v>131</v>
       </c>
       <c r="G12" s="22">
         <f t="shared" ref="G12:G14" si="2">IFERROR(F12/D12,0)</f>
-        <v>0.8833333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="5">
+      <c r="B13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="6">
         <f>'Datos CP'!D40</f>
         <v>169</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="6">
         <f>'Datos CP'!G40</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E13" s="22">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
+        <v>0.3136094675</v>
+      </c>
+      <c r="F13" s="6">
         <f>'Datos CP'!H40</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G13" s="22">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="5">
+      <c r="B14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="6">
         <f>'Datos CP'!D40</f>
         <v>169</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="6">
         <f>'Datos CP'!I40</f>
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="E14" s="22">
         <f t="shared" si="1"/>
-        <v>0.4142011834</v>
-      </c>
-      <c r="F14" s="5">
+        <v>0.798816568</v>
+      </c>
+      <c r="F14" s="6">
         <f>'Datos CP'!J40</f>
-        <v>60</v>
+        <v>133</v>
       </c>
       <c r="G14" s="22">
         <f t="shared" si="2"/>
-        <v>0.8571428571</v>
+        <v>0.9851851852</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="24" t="s">
-        <v>40</v>
+      <c r="B17" s="26" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="18">
@@ -1020,88 +993,88 @@
         <v>2</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="s">
-        <v>7</v>
+      <c r="B19" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="C19" s="22">
         <v>1.0</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="6">
         <f>SUMIFS('Datos CP'!$D$2:$D$39,'Datos CP'!$C$2:$C$39,B19)</f>
         <v>91</v>
       </c>
       <c r="E19" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$E$2:$E$39,'Datos CP'!$C$2:$C$39,B19)/D19,0)</f>
-        <v>0.4175824176</v>
+        <v>0.7142857143</v>
       </c>
       <c r="F19" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$G$2:$G$39,'Datos CP'!$C$2:$C$39,B19)/D19,0)</f>
-        <v>0</v>
+        <v>0.3186813187</v>
       </c>
       <c r="G19" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$I$2:$I$39,'Datos CP'!$C$2:$C$39,B19)/D19,0)</f>
-        <v>0.5054945055</v>
-      </c>
-      <c r="H19" s="5" t="str">
+        <v>0.7472527473</v>
+      </c>
+      <c r="H19" s="6" t="str">
         <f t="shared" ref="H19:H21" si="3">IF(AND(E19&gt;=C19,F19&gt;=C19,G19&gt;=C19),"Si","No")</f>
         <v>No</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="s">
-        <v>11</v>
+      <c r="B20" s="6" t="s">
+        <v>14</v>
       </c>
       <c r="C20" s="22">
         <v>0.75</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="6">
         <f>SUMIFS('Datos CP'!$D$2:$D$39,'Datos CP'!$C$2:$C$39,B20)</f>
         <v>75</v>
       </c>
       <c r="E20" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$E$2:$E$39,'Datos CP'!$C$2:$C$39,B20)/D20,0)</f>
-        <v>0.2533333333</v>
+        <v>0.84</v>
       </c>
       <c r="F20" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$G$2:$G$39,'Datos CP'!$C$2:$C$39,B20)/D20,0)</f>
-        <v>0</v>
+        <v>0.28</v>
       </c>
       <c r="G20" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$I$2:$I$39,'Datos CP'!$C$2:$C$39,B20)/D20,0)</f>
-        <v>0.28</v>
-      </c>
-      <c r="H20" s="5" t="str">
+        <v>0.8533333333</v>
+      </c>
+      <c r="H20" s="6" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="B21" s="5" t="s">
-        <v>13</v>
+      <c r="B21" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="C21" s="22">
         <v>0.75</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="6">
         <f>SUMIFS('Datos CP'!$D$2:$D$39,'Datos CP'!$C$2:$C$39,B21)</f>
         <v>3</v>
       </c>
@@ -1111,55 +1084,55 @@
       </c>
       <c r="F21" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$G$2:$G$39,'Datos CP'!$C$2:$C$39,B21)/D21,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="22">
         <f>IFERROR(SUMIFS('Datos CP'!$I$2:$I$39,'Datos CP'!$C$2:$C$39,B21)/D21,0)</f>
         <v>1</v>
       </c>
-      <c r="H21" s="5" t="str">
+      <c r="H21" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>No</v>
+        <v>Si</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="B24" s="24" t="s">
-        <v>57</v>
+      <c r="B24" s="26" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="B25" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>58</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="5">
+      <c r="B26" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="6">
         <f>Bugs!B5</f>
         <v>7</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="B27" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="5">
+      <c r="B27" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="6">
         <f>Bugs!B6</f>
         <v>5</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="B28" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="5">
+      <c r="B28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="6">
         <f>Bugs!B7</f>
         <v>2</v>
       </c>
@@ -2188,1396 +2161,1334 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="12">
+        <v>6.0</v>
+      </c>
+      <c r="E2" s="13">
+        <v>6.0</v>
+      </c>
+      <c r="F2" s="13">
+        <v>6.0</v>
+      </c>
+      <c r="G2" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H2" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I2" s="13">
+        <v>6.0</v>
+      </c>
+      <c r="J2" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="16"/>
+      <c r="B3" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="E3" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F3" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="G3" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H3" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I3" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="J3" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="16"/>
+      <c r="B4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="12">
+        <v>7.0</v>
+      </c>
+      <c r="E4" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="F4" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="G4" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H4" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I4" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="J4" s="13">
+        <v>6.0</v>
+      </c>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16"/>
+      <c r="B5" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16"/>
+      <c r="B6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="D6" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J6" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16"/>
+      <c r="B7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J7" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16"/>
+      <c r="B8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J8" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="18"/>
+      <c r="B9" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="12">
+        <v>7.0</v>
+      </c>
+      <c r="E10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J10" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16"/>
+      <c r="B11" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J11" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16"/>
+      <c r="B12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="13">
+        <v>5.0</v>
+      </c>
+      <c r="E12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J12" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16"/>
+      <c r="B13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="E13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J13" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="18"/>
+      <c r="B14" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="J14" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="14"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="12">
+        <v>7.0</v>
+      </c>
+      <c r="E15" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="F15" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="G15" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H15" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I15" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="J15" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16"/>
+      <c r="B16" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="E16" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="F16" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="G16" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H16" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I16" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="J16" s="13">
+        <v>7.0</v>
+      </c>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16"/>
+      <c r="B17" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="E17" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="F17" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="G17" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H17" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I17" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="J17" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="18"/>
+      <c r="B18" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="12">
+        <v>8.0</v>
+      </c>
+      <c r="E18" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="F18" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="G18" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H18" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I18" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="J18" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="E19" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="F19" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="G19" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H19" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I19" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="J19" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16"/>
+      <c r="B20" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="12">
+        <v>8.0</v>
+      </c>
+      <c r="E20" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="F20" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="G20" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H20" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I20" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="J20" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="16"/>
+      <c r="B21" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="12">
+        <v>9.0</v>
+      </c>
+      <c r="E21" s="13">
+        <v>9.0</v>
+      </c>
+      <c r="F21" s="13">
+        <v>9.0</v>
+      </c>
+      <c r="G21" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H21" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I21" s="13">
+        <v>9.0</v>
+      </c>
+      <c r="J21" s="13">
+        <v>9.0</v>
+      </c>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="18"/>
+      <c r="B22" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="12">
+        <v>8.0</v>
+      </c>
+      <c r="E22" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="F22" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="G22" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="H22" s="12">
+        <v>0.0</v>
+      </c>
+      <c r="I22" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="J22" s="13">
+        <v>8.0</v>
+      </c>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="F23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="G23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="H23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="I23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="J23" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="24"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="18"/>
+      <c r="B24" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="E24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="G24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="H24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="I24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="J24" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="25"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="F25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="H25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="I25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="J25" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="K25" s="14"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="25"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="16"/>
+      <c r="B26" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="F26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="H26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="I26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="J26" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="K26" s="14"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="25"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="16"/>
+      <c r="B27" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="F27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="G27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="H27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="I27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="J27" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K27" s="14"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="25"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="16"/>
+      <c r="B28" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="12">
+        <v>2.0</v>
+      </c>
+      <c r="E28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="F28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="H28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="I28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="J28" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="K28" s="14"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="25"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="18"/>
+      <c r="B29" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="14">
-        <v>6.0</v>
-      </c>
-      <c r="E2" s="15">
-        <v>6.0</v>
-      </c>
-      <c r="F2" s="15">
-        <v>6.0</v>
-      </c>
-      <c r="G2" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H2" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I2" s="15">
-        <v>6.0</v>
-      </c>
-      <c r="J2" s="16">
-        <v>5.0</v>
-      </c>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="20"/>
-      <c r="B3" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="14">
+      <c r="D29" s="12">
         <v>3.0</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E29" s="13">
         <v>3.0</v>
       </c>
-      <c r="F3" s="15">
+      <c r="F29" s="13">
         <v>3.0</v>
       </c>
-      <c r="G3" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H3" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I3" s="15">
+      <c r="G29" s="13">
         <v>3.0</v>
       </c>
-      <c r="J3" s="16">
+      <c r="H29" s="13">
         <v>3.0</v>
       </c>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="20"/>
-      <c r="B4" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="14">
-        <v>7.0</v>
-      </c>
-      <c r="E4" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="F4" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H4" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I4" s="15">
-        <v>7.0</v>
-      </c>
-      <c r="J4" s="16">
-        <v>6.0</v>
-      </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="20"/>
-      <c r="B5" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="14">
+      <c r="I29" s="13">
         <v>3.0</v>
       </c>
-      <c r="E5" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F5" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G5" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H5" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I5" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J5" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="20"/>
-      <c r="B6" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="14">
+      <c r="J29" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="K29" s="14"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="25"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="F30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="G30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="H30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="I30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="J30" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="25"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="16"/>
+      <c r="B31" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E31" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F31" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="G31" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="H31" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="I31" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="J31" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="24"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="18"/>
+      <c r="B32" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="12">
         <v>2.0</v>
       </c>
-      <c r="E6" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F6" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G6" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H6" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I6" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J6" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="20"/>
-      <c r="B7" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="14">
+      <c r="E32" s="13">
         <v>2.0</v>
       </c>
-      <c r="E7" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F7" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G7" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H7" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I7" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J7" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="20"/>
-      <c r="B8" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="14">
+      <c r="F32" s="13">
         <v>2.0</v>
       </c>
-      <c r="E8" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G8" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H8" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I8" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J8" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="25"/>
-      <c r="B9" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="14">
+      <c r="G32" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="H32" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="I32" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="J32" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="24"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="12">
         <v>4.0</v>
       </c>
-      <c r="E9" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F9" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H9" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I9" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J9" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="18"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="14">
-        <v>7.0</v>
-      </c>
-      <c r="E10" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F10" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G10" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H10" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I10" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J10" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="20"/>
-      <c r="B11" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="14">
+      <c r="E33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="F33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="G33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="H33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="I33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="J33" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="25"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="16"/>
+      <c r="B34" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="12">
+        <v>3.0</v>
+      </c>
+      <c r="E34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="G34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="H34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="I34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="J34" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="K34" s="27"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="28"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="16"/>
+      <c r="B35" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="12">
         <v>2.0</v>
       </c>
-      <c r="E11" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F11" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G11" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H11" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I11" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J11" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="20"/>
-      <c r="B12" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="15">
-        <v>5.0</v>
-      </c>
-      <c r="E12" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G12" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H12" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I12" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J12" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="20"/>
-      <c r="B13" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="14">
+      <c r="E35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="F35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="H35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="I35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="J35" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="K35" s="14"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="25"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="18"/>
+      <c r="B36" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="12">
+        <v>4.0</v>
+      </c>
+      <c r="E36" s="13">
         <v>3.0</v>
       </c>
-      <c r="E13" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F13" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G13" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H13" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I13" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J13" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="18"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="25"/>
-      <c r="B14" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="14">
+      <c r="F36" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="G36" s="13">
         <v>4.0</v>
       </c>
-      <c r="E14" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F14" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G14" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H14" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I14" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J14" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="14">
-        <v>7.0</v>
-      </c>
-      <c r="E15" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F15" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G15" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H15" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I15" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J15" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="20"/>
-      <c r="B16" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="15">
-        <v>7.0</v>
-      </c>
-      <c r="E16" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F16" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G16" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H16" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I16" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J16" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="20"/>
-      <c r="B17" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="15">
-        <v>10.0</v>
-      </c>
-      <c r="E17" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F17" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G17" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H17" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I17" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J17" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="25"/>
-      <c r="B18" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="14">
-        <v>8.0</v>
-      </c>
-      <c r="E18" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F18" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G18" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H18" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I18" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J18" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="15">
-        <v>8.0</v>
-      </c>
-      <c r="E19" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F19" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G19" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H19" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I19" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J19" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="20"/>
-      <c r="B20" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="14">
-        <v>8.0</v>
-      </c>
-      <c r="E20" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F20" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G20" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H20" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I20" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J20" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="20"/>
-      <c r="B21" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="14">
-        <v>9.0</v>
-      </c>
-      <c r="E21" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F21" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G21" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H21" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I21" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J21" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="25"/>
-      <c r="B22" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="14">
-        <v>8.0</v>
-      </c>
-      <c r="E22" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="F22" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="G22" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H22" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I22" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="J22" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="14">
+      <c r="H36" s="13">
         <v>4.0</v>
       </c>
-      <c r="E23" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F23" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G23" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H23" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I23" s="15">
+      <c r="I36" s="13">
         <v>4.0</v>
       </c>
-      <c r="J23" s="16">
+      <c r="J36" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="25"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="12">
         <v>3.0</v>
       </c>
-      <c r="K23" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="L23" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M23" s="27" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="25"/>
-      <c r="B24" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="15">
+      <c r="E37" s="13">
         <v>3.0</v>
       </c>
-      <c r="E24" s="15">
+      <c r="F37" s="13">
         <v>3.0</v>
       </c>
-      <c r="F24" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G24" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H24" s="15">
-        <v>0.0</v>
-      </c>
-      <c r="I24" s="15">
+      <c r="G37" s="13">
         <v>3.0</v>
       </c>
-      <c r="J24" s="16">
+      <c r="H37" s="13">
         <v>3.0</v>
       </c>
-      <c r="K24" s="18"/>
-      <c r="L24" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M24" s="28"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E25" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F25" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G25" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H25" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I25" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="J25" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K25" s="18"/>
-      <c r="L25" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M25" s="28"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="20"/>
-      <c r="B26" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E26" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F26" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G26" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H26" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I26" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="J26" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K26" s="18"/>
-      <c r="L26" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M26" s="28"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="20"/>
-      <c r="B27" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="14">
+      <c r="I37" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="J37" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="24"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="16"/>
+      <c r="B38" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="12">
         <v>4.0</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E38" s="13">
         <v>4.0</v>
       </c>
-      <c r="F27" s="15">
+      <c r="F38" s="13">
         <v>4.0</v>
       </c>
-      <c r="G27" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H27" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I27" s="15">
+      <c r="G38" s="13">
         <v>4.0</v>
       </c>
-      <c r="J27" s="16">
+      <c r="H38" s="13">
         <v>4.0</v>
       </c>
-      <c r="K27" s="18"/>
-      <c r="L27" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M27" s="28"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="20"/>
-      <c r="B28" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E28" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F28" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G28" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H28" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I28" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="J28" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K28" s="18"/>
-      <c r="L28" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M28" s="28"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="25"/>
-      <c r="B29" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="E29" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="F29" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="G29" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H29" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I29" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="J29" s="16">
-        <v>3.0</v>
-      </c>
-      <c r="K29" s="18"/>
-      <c r="L29" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M29" s="28"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="14">
+      <c r="I38" s="13">
         <v>4.0</v>
       </c>
-      <c r="E30" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="F30" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="G30" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H30" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I30" s="15">
+      <c r="J38" s="13">
         <v>4.0</v>
       </c>
-      <c r="J30" s="16">
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="24"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="18"/>
+      <c r="B39" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="12">
         <v>4.0</v>
       </c>
-      <c r="K30" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="L30" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M30" s="28"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="20"/>
-      <c r="B31" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="14">
+      <c r="E39" s="13">
         <v>4.0</v>
       </c>
-      <c r="E31" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="F31" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="G31" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H31" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I31" s="15">
+      <c r="F39" s="13">
         <v>4.0</v>
       </c>
-      <c r="J31" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K31" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="L31" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M31" s="27" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="25"/>
-      <c r="B32" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E32" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F32" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G32" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H32" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I32" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="J32" s="16">
-        <v>0.0</v>
-      </c>
-      <c r="K32" s="18"/>
-      <c r="L32" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M32" s="27" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="14">
+      <c r="G39" s="13">
         <v>4.0</v>
       </c>
-      <c r="E33" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F33" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G33" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H33" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I33" s="15">
+      <c r="H39" s="13">
         <v>4.0</v>
       </c>
-      <c r="J33" s="16">
+      <c r="I39" s="13">
         <v>4.0</v>
       </c>
-      <c r="K33" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="L33" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M33" s="28"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="20"/>
-      <c r="B34" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="E34" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="F34" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G34" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H34" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I34" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="J34" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K34" s="29"/>
-      <c r="L34" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M34" s="30" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="20"/>
-      <c r="B35" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="14">
-        <v>2.0</v>
-      </c>
-      <c r="E35" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F35" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="G35" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H35" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I35" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="J35" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K35" s="18"/>
-      <c r="L35" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M35" s="28"/>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="25"/>
-      <c r="B36" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="14">
+      <c r="J39" s="13">
         <v>4.0</v>
       </c>
-      <c r="E36" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="F36" s="15">
-        <v>2.0</v>
-      </c>
-      <c r="G36" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H36" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I36" s="15">
-        <v>4.0</v>
-      </c>
-      <c r="J36" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="K36" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="L36" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M36" s="28"/>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="B37" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C37" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="14">
-        <v>3.0</v>
-      </c>
-      <c r="E37" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="F37" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="G37" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H37" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I37" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="J37" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M37" s="27" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="20"/>
-      <c r="B38" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38" s="14">
-        <v>4.0</v>
-      </c>
-      <c r="E38" s="15">
-        <v>4.0</v>
-      </c>
-      <c r="F38" s="15">
-        <v>3.0</v>
-      </c>
-      <c r="G38" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H38" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I38" s="15">
-        <v>4.0</v>
-      </c>
-      <c r="J38" s="16">
-        <v>3.0</v>
-      </c>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M38" s="27" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="25"/>
-      <c r="B39" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="14">
-        <v>4.0</v>
-      </c>
-      <c r="E39" s="15">
-        <v>4.0</v>
-      </c>
-      <c r="F39" s="15">
-        <v>1.0</v>
-      </c>
-      <c r="G39" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="H39" s="14">
-        <v>0.0</v>
-      </c>
-      <c r="I39" s="15">
-        <v>4.0</v>
-      </c>
-      <c r="J39" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="K39" s="18"/>
-      <c r="L39" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="M39" s="28"/>
+      <c r="K39" s="14"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="25"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="B40" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C40" s="31"/>
-      <c r="D40" s="32">
+      <c r="B40" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="29"/>
+      <c r="D40" s="30">
         <f t="shared" ref="D40:J40" si="1">SUM(D2:D39)</f>
         <v>169</v>
       </c>
-      <c r="E40" s="32">
+      <c r="E40" s="30">
         <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="F40" s="32">
+        <v>131</v>
+      </c>
+      <c r="F40" s="30">
+        <f t="shared" si="1"/>
+        <v>131</v>
+      </c>
+      <c r="G40" s="30">
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
-      <c r="G40" s="32">
+      <c r="H40" s="30">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H40" s="32">
+        <v>53</v>
+      </c>
+      <c r="I40" s="30">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I40" s="32">
+        <v>135</v>
+      </c>
+      <c r="J40" s="30">
         <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-      <c r="J40" s="32">
-        <f t="shared" si="1"/>
-        <v>60</v>
+        <v>133</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
@@ -4555,7 +4466,8 @@
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -4579,41 +4491,41 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="6">
+      <c r="A5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="8">
         <v>7.0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="6">
+      <c r="A6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="8">
         <v>5.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="6">
         <v>2.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="9">
+      <c r="A8" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="10">
         <f>SUM(B5:B7)</f>
         <v>14</v>
       </c>

</xml_diff>